<commit_message>
PAMPALO.HE CR:nc|high. + Excel + D&A
</commit_message>
<xml_diff>
--- a/data/hex_xlsx/PAMPALO.HE.xlsx
+++ b/data/hex_xlsx/PAMPALO.HE.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="266">
   <si>
     <t>Company Fundamentals - Income Statement</t>
   </si>
@@ -154,6 +154,9 @@
   </si>
   <si>
     <t>Depreciation and impairment losses</t>
+  </si>
+  <si>
+    <t>Depreciation</t>
   </si>
   <si>
     <t>Impairment - Fixed Assets</t>
@@ -939,7 +942,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1005,6 +1008,9 @@
     </xf>
     <xf borderId="3" fillId="0" fontId="3" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="3" fillId="0" fontId="6" numFmtId="4" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -1646,7 +1652,9 @@
       <c r="C27" s="21">
         <v>37.18</v>
       </c>
-      <c r="D27" s="16"/>
+      <c r="D27" s="21">
+        <v>26.24</v>
+      </c>
       <c r="E27" s="21">
         <v>83.78</v>
       </c>
@@ -1655,11 +1663,17 @@
       </c>
     </row>
     <row r="28" ht="15.0" customHeight="1">
-      <c r="A28" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="B28" s="16"/>
-      <c r="C28" s="16"/>
+      <c r="A28" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="B28" s="16">
+        <f t="shared" ref="B28:C28" si="1">B27</f>
+        <v>101.81</v>
+      </c>
+      <c r="C28" s="16">
+        <f t="shared" si="1"/>
+        <v>37.18</v>
+      </c>
       <c r="D28" s="21">
         <v>26.24</v>
       </c>
@@ -1672,7 +1686,7 @@
     </row>
     <row r="29" ht="15.0" customHeight="1">
       <c r="A29" s="14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
@@ -1688,7 +1702,7 @@
     </row>
     <row r="30" ht="15.0" customHeight="1">
       <c r="A30" s="14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B30" s="16"/>
       <c r="C30" s="16"/>
@@ -1700,7 +1714,7 @@
     </row>
     <row r="31" ht="15.0" customHeight="1">
       <c r="A31" s="14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B31" s="16"/>
       <c r="C31" s="16"/>
@@ -1712,7 +1726,7 @@
     </row>
     <row r="32" ht="15.0" customHeight="1">
       <c r="A32" s="17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B32" s="18">
         <v>443.53</v>
@@ -1732,7 +1746,7 @@
     </row>
     <row r="33" ht="15.0" customHeight="1">
       <c r="A33" s="14" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
@@ -1746,27 +1760,27 @@
     </row>
     <row r="34" ht="15.0" customHeight="1">
       <c r="A34" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="B34" s="22">
+        <v>51</v>
+      </c>
+      <c r="B34" s="23">
         <v>88.94</v>
       </c>
-      <c r="C34" s="22">
+      <c r="C34" s="23">
         <v>30.21</v>
       </c>
-      <c r="D34" s="23">
+      <c r="D34" s="24">
         <v>-34.22</v>
       </c>
-      <c r="E34" s="24">
+      <c r="E34" s="25">
         <v>-148.38</v>
       </c>
-      <c r="F34" s="24">
+      <c r="F34" s="25">
         <v>-255.06</v>
       </c>
     </row>
     <row r="35" ht="15.0" customHeight="1">
       <c r="A35" s="14" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B35" s="21">
         <v>8.19</v>
@@ -1786,7 +1800,7 @@
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="14" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B36" s="16"/>
       <c r="C36" s="16">
@@ -1804,7 +1818,7 @@
     </row>
     <row r="37" ht="15.0" customHeight="1">
       <c r="A37" s="14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="21">
@@ -1818,7 +1832,7 @@
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="14" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B38" s="16"/>
       <c r="C38" s="16"/>
@@ -1832,7 +1846,7 @@
     </row>
     <row r="39" ht="15.0" customHeight="1">
       <c r="A39" s="14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B39" s="20">
         <v>-59.68</v>
@@ -1852,7 +1866,7 @@
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B40" s="16"/>
       <c r="C40" s="20">
@@ -1866,7 +1880,7 @@
     </row>
     <row r="41" ht="15.0" customHeight="1">
       <c r="A41" s="14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="20">
@@ -1884,7 +1898,7 @@
     </row>
     <row r="42" ht="15.0" customHeight="1">
       <c r="A42" s="14" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B42" s="16"/>
       <c r="C42" s="16">
@@ -1902,7 +1916,7 @@
     </row>
     <row r="43" ht="15.0" customHeight="1">
       <c r="A43" s="14" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B43" s="16"/>
       <c r="C43" s="20">
@@ -1920,27 +1934,27 @@
     </row>
     <row r="44" ht="15.0" customHeight="1">
       <c r="A44" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="B44" s="23">
+        <v>61</v>
+      </c>
+      <c r="B44" s="24">
         <v>-51.49</v>
       </c>
-      <c r="C44" s="23">
+      <c r="C44" s="24">
         <v>-26.73</v>
       </c>
-      <c r="D44" s="23">
+      <c r="D44" s="24">
         <v>-26.24</v>
       </c>
-      <c r="E44" s="23">
+      <c r="E44" s="24">
         <v>-27.25</v>
       </c>
-      <c r="F44" s="23">
+      <c r="F44" s="24">
         <v>-5.08</v>
       </c>
     </row>
     <row r="45" ht="15.0" customHeight="1">
       <c r="A45" s="14" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="21">
@@ -1956,27 +1970,27 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="A46" s="17" t="s">
-        <v>62</v>
-      </c>
-      <c r="B46" s="22">
+        <v>63</v>
+      </c>
+      <c r="B46" s="23">
         <v>37.45</v>
       </c>
-      <c r="C46" s="22">
+      <c r="C46" s="23">
         <v>4.65</v>
       </c>
-      <c r="D46" s="23">
+      <c r="D46" s="24">
         <v>-60.46</v>
       </c>
-      <c r="E46" s="24">
+      <c r="E46" s="25">
         <v>-176.64</v>
       </c>
-      <c r="F46" s="24">
+      <c r="F46" s="25">
         <v>-261.16</v>
       </c>
     </row>
     <row r="47" ht="15.0" customHeight="1">
       <c r="A47" s="14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B47" s="20">
         <v>-47.98</v>
@@ -1996,7 +2010,7 @@
     </row>
     <row r="48" ht="15.0" customHeight="1">
       <c r="A48" s="14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B48" s="16"/>
       <c r="C48" s="21">
@@ -2008,12 +2022,12 @@
     </row>
     <row r="49" ht="15.0" customHeight="1">
       <c r="A49" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="B49" s="23">
+        <v>66</v>
+      </c>
+      <c r="B49" s="24">
         <v>-47.98</v>
       </c>
-      <c r="C49" s="22">
+      <c r="C49" s="23">
         <v>1.16</v>
       </c>
       <c r="D49" s="19">
@@ -2028,67 +2042,67 @@
     </row>
     <row r="50" ht="15.0" customHeight="1">
       <c r="A50" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="B50" s="22">
+        <v>67</v>
+      </c>
+      <c r="B50" s="23">
         <v>85.43</v>
       </c>
-      <c r="C50" s="22">
+      <c r="C50" s="23">
         <v>3.49</v>
       </c>
-      <c r="D50" s="23">
+      <c r="D50" s="24">
         <v>-60.46</v>
       </c>
-      <c r="E50" s="24">
+      <c r="E50" s="25">
         <v>-176.64</v>
       </c>
-      <c r="F50" s="24">
+      <c r="F50" s="25">
         <v>-261.16</v>
       </c>
     </row>
     <row r="51" ht="15.0" customHeight="1">
       <c r="A51" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="B51" s="22">
+        <v>68</v>
+      </c>
+      <c r="B51" s="23">
         <v>85.43</v>
       </c>
-      <c r="C51" s="22">
+      <c r="C51" s="23">
         <v>3.49</v>
       </c>
-      <c r="D51" s="23">
+      <c r="D51" s="24">
         <v>-60.46</v>
       </c>
-      <c r="E51" s="24">
+      <c r="E51" s="25">
         <v>-176.64</v>
       </c>
-      <c r="F51" s="24">
+      <c r="F51" s="25">
         <v>-261.16</v>
       </c>
     </row>
     <row r="52" ht="15.0" customHeight="1">
       <c r="A52" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="B52" s="22">
+        <v>69</v>
+      </c>
+      <c r="B52" s="23">
         <v>85.43</v>
       </c>
-      <c r="C52" s="22">
+      <c r="C52" s="23">
         <v>3.49</v>
       </c>
-      <c r="D52" s="23">
+      <c r="D52" s="24">
         <v>-60.46</v>
       </c>
-      <c r="E52" s="24">
+      <c r="E52" s="25">
         <v>-176.64</v>
       </c>
-      <c r="F52" s="24">
+      <c r="F52" s="25">
         <v>-261.16</v>
       </c>
     </row>
     <row r="53" ht="15.0" customHeight="1">
       <c r="A53" s="14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B53" s="16"/>
       <c r="C53" s="21">
@@ -2100,7 +2114,7 @@
     </row>
     <row r="54" ht="15.0" customHeight="1">
       <c r="A54" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B54" s="16"/>
       <c r="C54" s="21">
@@ -2112,10 +2126,10 @@
     </row>
     <row r="55" ht="15.0" customHeight="1">
       <c r="A55" s="17" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B55" s="19"/>
-      <c r="C55" s="22">
+      <c r="C55" s="23">
         <v>13.94</v>
       </c>
       <c r="D55" s="19"/>
@@ -2124,7 +2138,7 @@
     </row>
     <row r="56" ht="15.0" customHeight="1">
       <c r="A56" s="14" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B56" s="16"/>
       <c r="C56" s="21">
@@ -2136,10 +2150,10 @@
     </row>
     <row r="57" ht="15.0" customHeight="1">
       <c r="A57" s="17" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B57" s="19"/>
-      <c r="C57" s="22">
+      <c r="C57" s="23">
         <v>17.43</v>
       </c>
       <c r="D57" s="19"/>
@@ -2148,7 +2162,7 @@
     </row>
     <row r="58" ht="15.0" customHeight="1">
       <c r="A58" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B58" s="16"/>
       <c r="C58" s="21">
@@ -2160,7 +2174,7 @@
     </row>
     <row r="59" ht="15.0" customHeight="1">
       <c r="A59" s="14" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B59" s="16"/>
       <c r="C59" s="21">
@@ -2178,7 +2192,7 @@
     </row>
     <row r="60" ht="15.0" customHeight="1">
       <c r="A60" s="14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B60" s="16"/>
       <c r="C60" s="15">
@@ -2196,7 +2210,7 @@
     </row>
     <row r="61" ht="15.0" customHeight="1">
       <c r="A61" s="14" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B61" s="16"/>
       <c r="C61" s="21">
@@ -2208,7 +2222,7 @@
     </row>
     <row r="62" ht="15.0" customHeight="1">
       <c r="A62" s="14" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B62" s="16"/>
       <c r="C62" s="15">
@@ -2226,7 +2240,7 @@
     </row>
     <row r="63" ht="15.0" customHeight="1">
       <c r="A63" s="14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B63" s="15">
         <v>101.81</v>
@@ -2244,7 +2258,7 @@
     </row>
     <row r="64" ht="15.0" customHeight="1">
       <c r="A64" s="14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B64" s="16"/>
       <c r="C64" s="21">
@@ -2256,7 +2270,7 @@
     </row>
     <row r="65" ht="15.0" customHeight="1">
       <c r="A65" s="14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B65" s="16"/>
       <c r="C65" s="16">
@@ -2268,7 +2282,7 @@
     </row>
     <row r="66" ht="15.0" customHeight="1">
       <c r="A66" s="14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B66" s="16"/>
       <c r="C66" s="21">
@@ -2280,7 +2294,7 @@
     </row>
     <row r="67" ht="15.0" customHeight="1">
       <c r="A67" s="14" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B67" s="16"/>
       <c r="C67" s="16">
@@ -2298,7 +2312,7 @@
     </row>
     <row r="68" ht="15.0" customHeight="1">
       <c r="A68" s="14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B68" s="21">
         <v>85.43</v>
@@ -2309,16 +2323,16 @@
       <c r="D68" s="20">
         <v>-60.46</v>
       </c>
-      <c r="E68" s="25">
+      <c r="E68" s="26">
         <v>-176.64</v>
       </c>
-      <c r="F68" s="25">
+      <c r="F68" s="26">
         <v>-261.16</v>
       </c>
     </row>
     <row r="69" ht="15.0" customHeight="1">
       <c r="A69" s="14" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B69" s="21">
         <v>85.43</v>
@@ -2329,16 +2343,16 @@
       <c r="D69" s="20">
         <v>-60.46</v>
       </c>
-      <c r="E69" s="25">
+      <c r="E69" s="26">
         <v>-176.64</v>
       </c>
-      <c r="F69" s="25">
+      <c r="F69" s="26">
         <v>-261.16</v>
       </c>
     </row>
     <row r="70" ht="15.0" customHeight="1">
       <c r="A70" s="14" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B70" s="21">
         <v>8.19</v>
@@ -2358,7 +2372,7 @@
     </row>
     <row r="71" ht="15.0" customHeight="1">
       <c r="A71" s="14" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B71" s="21">
         <v>8.19</v>
@@ -2378,7 +2392,7 @@
     </row>
     <row r="72" ht="15.0" customHeight="1">
       <c r="A72" s="14" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B72" s="21">
         <v>7.02</v>
@@ -2398,7 +2412,7 @@
     </row>
     <row r="73" ht="15.0" customHeight="1">
       <c r="A73" s="14" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B73" s="21">
         <v>7.02</v>
@@ -2418,7 +2432,7 @@
     </row>
     <row r="74" ht="15.0" customHeight="1">
       <c r="A74" s="14" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B74" s="21">
         <v>12.25</v>
@@ -2438,7 +2452,7 @@
     </row>
     <row r="75" ht="15.0" customHeight="1">
       <c r="A75" s="14" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B75" s="21">
         <v>11.19</v>
@@ -2458,7 +2472,7 @@
     </row>
     <row r="76" ht="15.0" customHeight="1">
       <c r="A76" s="14" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B76" s="21">
         <v>11.19</v>
@@ -2478,7 +2492,7 @@
     </row>
     <row r="77" ht="15.0" customHeight="1">
       <c r="A77" s="14" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B77" s="21">
         <v>12.25</v>
@@ -2498,7 +2512,7 @@
     </row>
     <row r="78" ht="15.0" customHeight="1">
       <c r="A78" s="14" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B78" s="21">
         <v>8.19</v>
@@ -2518,7 +2532,7 @@
     </row>
     <row r="79" ht="15.0" customHeight="1">
       <c r="A79" s="14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B79" s="21">
         <v>7.02</v>
@@ -2538,7 +2552,7 @@
     </row>
     <row r="80" ht="15.0" customHeight="1">
       <c r="A80" s="14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B80" s="21">
         <v>85.43</v>
@@ -2549,16 +2563,16 @@
       <c r="D80" s="20">
         <v>-60.46</v>
       </c>
-      <c r="E80" s="25">
+      <c r="E80" s="26">
         <v>-176.64</v>
       </c>
-      <c r="F80" s="25">
+      <c r="F80" s="26">
         <v>-261.16</v>
       </c>
     </row>
     <row r="81" ht="15.0" customHeight="1">
       <c r="A81" s="14" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B81" s="21">
         <v>85.43</v>
@@ -2569,16 +2583,16 @@
       <c r="D81" s="20">
         <v>-60.46</v>
       </c>
-      <c r="E81" s="25">
+      <c r="E81" s="26">
         <v>-176.64</v>
       </c>
-      <c r="F81" s="25">
+      <c r="F81" s="26">
         <v>-261.16</v>
       </c>
     </row>
     <row r="82" ht="15.0" customHeight="1">
       <c r="A82" s="14" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B82" s="21">
         <v>8.19</v>
@@ -2598,7 +2612,7 @@
     </row>
     <row r="83" ht="15.0" customHeight="1">
       <c r="A83" s="14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B83" s="21">
         <v>7.02</v>
@@ -2618,7 +2632,7 @@
     </row>
     <row r="84" ht="15.0" customHeight="1">
       <c r="A84" s="14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B84" s="21">
         <v>1.0</v>
@@ -2638,7 +2652,7 @@
     </row>
     <row r="85" ht="15.0" customHeight="1">
       <c r="A85" s="14" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B85" s="21">
         <v>85.43</v>
@@ -2649,16 +2663,16 @@
       <c r="D85" s="20">
         <v>-60.46</v>
       </c>
-      <c r="E85" s="25">
+      <c r="E85" s="26">
         <v>-176.64</v>
       </c>
-      <c r="F85" s="25">
+      <c r="F85" s="26">
         <v>-261.16</v>
       </c>
     </row>
     <row r="86" ht="15.0" customHeight="1">
       <c r="A86" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B86" s="21">
         <v>85.43</v>
@@ -2669,16 +2683,16 @@
       <c r="D86" s="20">
         <v>-60.46</v>
       </c>
-      <c r="E86" s="25">
+      <c r="E86" s="26">
         <v>-176.64</v>
       </c>
-      <c r="F86" s="25">
+      <c r="F86" s="26">
         <v>-261.16</v>
       </c>
     </row>
     <row r="87" ht="15.0" customHeight="1">
       <c r="A87" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B87" s="21">
         <v>1.0</v>
@@ -3631,7 +3645,7 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3796,19 +3810,19 @@
         <v>27</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="16" ht="15.0" customHeight="1" outlineLevel="1">
@@ -3823,7 +3837,7 @@
     </row>
     <row r="18">
       <c r="A18" s="12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -3853,7 +3867,7 @@
     </row>
     <row r="20" ht="15.0" customHeight="1">
       <c r="A20" s="14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B20" s="15">
         <v>361.51</v>
@@ -3873,7 +3887,7 @@
     </row>
     <row r="21" ht="15.0" customHeight="1">
       <c r="A21" s="14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B21" s="16"/>
       <c r="C21" s="15">
@@ -3885,10 +3899,10 @@
     </row>
     <row r="22" ht="15.0" customHeight="1">
       <c r="A22" s="14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B22" s="16"/>
-      <c r="C22" s="25">
+      <c r="C22" s="26">
         <v>-217.69</v>
       </c>
       <c r="D22" s="16"/>
@@ -3897,7 +3911,7 @@
     </row>
     <row r="23" ht="15.0" customHeight="1">
       <c r="A23" s="14" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B23" s="16"/>
       <c r="C23" s="21">
@@ -3909,7 +3923,7 @@
     </row>
     <row r="24" ht="15.0" customHeight="1">
       <c r="A24" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B24" s="21">
         <v>15.36</v>
@@ -3925,7 +3939,7 @@
     </row>
     <row r="25" ht="15.0" customHeight="1">
       <c r="A25" s="14" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B25" s="16"/>
       <c r="C25" s="21">
@@ -3937,7 +3951,7 @@
     </row>
     <row r="26" ht="15.0" customHeight="1">
       <c r="A26" s="14" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B26" s="16"/>
       <c r="C26" s="20">
@@ -3949,7 +3963,7 @@
     </row>
     <row r="27" ht="15.0" customHeight="1">
       <c r="A27" s="14" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B27" s="15">
         <v>226.83</v>
@@ -3969,7 +3983,7 @@
     </row>
     <row r="28" ht="15.0" customHeight="1">
       <c r="A28" s="14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B28" s="16"/>
       <c r="C28" s="15">
@@ -3981,10 +3995,10 @@
     </row>
     <row r="29" ht="15.0" customHeight="1">
       <c r="A29" s="14" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B29" s="16"/>
-      <c r="C29" s="25">
+      <c r="C29" s="26">
         <v>-290.64</v>
       </c>
       <c r="D29" s="16"/>
@@ -3993,7 +4007,7 @@
     </row>
     <row r="30" ht="15.0" customHeight="1">
       <c r="A30" s="14" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B30" s="16"/>
       <c r="C30" s="21">
@@ -4005,7 +4019,7 @@
     </row>
     <row r="31" ht="15.0" customHeight="1">
       <c r="A31" s="14" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B31" s="21">
         <v>38.99</v>
@@ -4021,7 +4035,7 @@
     </row>
     <row r="32" ht="15.0" customHeight="1">
       <c r="A32" s="14" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B32" s="16"/>
       <c r="C32" s="21">
@@ -4033,7 +4047,7 @@
     </row>
     <row r="33" ht="15.0" customHeight="1">
       <c r="A33" s="14" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="20">
@@ -4045,7 +4059,7 @@
     </row>
     <row r="34" ht="15.0" customHeight="1">
       <c r="A34" s="14" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B34" s="21">
         <v>3.54</v>
@@ -4065,7 +4079,7 @@
     </row>
     <row r="35" ht="15.0" customHeight="1">
       <c r="A35" s="14" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B35" s="16"/>
       <c r="C35" s="21">
@@ -4077,7 +4091,7 @@
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="14" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B36" s="16"/>
       <c r="C36" s="16">
@@ -4089,7 +4103,7 @@
     </row>
     <row r="37" ht="15.0" customHeight="1">
       <c r="A37" s="14" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B37" s="21">
         <v>29.54</v>
@@ -4109,7 +4123,7 @@
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="14" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B38" s="16"/>
       <c r="C38" s="15">
@@ -4121,10 +4135,10 @@
     </row>
     <row r="39" ht="15.0" customHeight="1">
       <c r="A39" s="14" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B39" s="16"/>
-      <c r="C39" s="25">
+      <c r="C39" s="26">
         <v>-117.67</v>
       </c>
       <c r="D39" s="16"/>
@@ -4133,7 +4147,7 @@
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="14" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B40" s="21">
         <v>63.8</v>
@@ -4153,7 +4167,7 @@
     </row>
     <row r="41" ht="15.0" customHeight="1">
       <c r="A41" s="14" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="15">
@@ -4165,10 +4179,10 @@
     </row>
     <row r="42" ht="15.0" customHeight="1">
       <c r="A42" s="14" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B42" s="16"/>
-      <c r="C42" s="25">
+      <c r="C42" s="26">
         <v>-275.35</v>
       </c>
       <c r="D42" s="16"/>
@@ -4177,7 +4191,7 @@
     </row>
     <row r="43" ht="15.0" customHeight="1">
       <c r="A43" s="14" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B43" s="21">
         <v>7.09</v>
@@ -4193,7 +4207,7 @@
     </row>
     <row r="44" ht="15.0" customHeight="1">
       <c r="A44" s="14" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B44" s="16"/>
       <c r="C44" s="21">
@@ -4205,7 +4219,7 @@
     </row>
     <row r="45" ht="15.0" customHeight="1">
       <c r="A45" s="14" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="16">
@@ -4217,7 +4231,7 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="A46" s="14" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B46" s="21">
         <v>10.63</v>
@@ -4237,7 +4251,7 @@
     </row>
     <row r="47" ht="15.0" customHeight="1">
       <c r="A47" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B47" s="21">
         <v>50.8</v>
@@ -4249,7 +4263,7 @@
     </row>
     <row r="48" ht="15.0" customHeight="1">
       <c r="A48" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B48" s="16"/>
       <c r="C48" s="16"/>
@@ -4263,7 +4277,7 @@
     </row>
     <row r="49" ht="15.0" customHeight="1">
       <c r="A49" s="17" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B49" s="18">
         <v>808.08</v>
@@ -4283,7 +4297,7 @@
     </row>
     <row r="50" ht="15.0" customHeight="1">
       <c r="A50" s="14" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B50" s="21">
         <v>13.0</v>
@@ -4303,7 +4317,7 @@
     </row>
     <row r="51" ht="15.0" customHeight="1">
       <c r="A51" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B51" s="16"/>
       <c r="C51" s="21">
@@ -4315,7 +4329,7 @@
     </row>
     <row r="52" ht="15.0" customHeight="1">
       <c r="A52" s="14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B52" s="16"/>
       <c r="C52" s="21">
@@ -4327,7 +4341,7 @@
     </row>
     <row r="53" ht="15.0" customHeight="1">
       <c r="A53" s="14" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B53" s="16"/>
       <c r="C53" s="21">
@@ -4339,7 +4353,7 @@
     </row>
     <row r="54" ht="15.0" customHeight="1">
       <c r="A54" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B54" s="16"/>
       <c r="C54" s="21">
@@ -4351,7 +4365,7 @@
     </row>
     <row r="55" ht="15.0" customHeight="1">
       <c r="A55" s="14" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B55" s="21">
         <v>90.97</v>
@@ -4371,7 +4385,7 @@
     </row>
     <row r="56" ht="15.0" customHeight="1">
       <c r="A56" s="14" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B56" s="16">
         <v>0.0</v>
@@ -4391,7 +4405,7 @@
     </row>
     <row r="57" ht="15.0" customHeight="1">
       <c r="A57" s="14" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B57" s="21">
         <v>2.36</v>
@@ -4411,7 +4425,7 @@
     </row>
     <row r="58" ht="15.0" customHeight="1">
       <c r="A58" s="14" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B58" s="21">
         <v>46.07</v>
@@ -4431,7 +4445,7 @@
     </row>
     <row r="59" ht="15.0" customHeight="1">
       <c r="A59" s="14" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B59" s="21">
         <v>1.18</v>
@@ -4447,27 +4461,27 @@
     </row>
     <row r="60" ht="15.0" customHeight="1">
       <c r="A60" s="17" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B60" s="18">
         <v>153.58</v>
       </c>
-      <c r="C60" s="22">
+      <c r="C60" s="23">
         <v>67.07</v>
       </c>
-      <c r="D60" s="22">
+      <c r="D60" s="23">
         <v>40.27</v>
       </c>
-      <c r="E60" s="22">
+      <c r="E60" s="23">
         <v>63.95</v>
       </c>
-      <c r="F60" s="22">
+      <c r="F60" s="23">
         <v>38.04</v>
       </c>
     </row>
     <row r="61" ht="15.0" customHeight="1">
       <c r="A61" s="14" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B61" s="15">
         <v>128.77</v>
@@ -4479,7 +4493,7 @@
     </row>
     <row r="62" ht="15.0" customHeight="1">
       <c r="A62" s="14" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B62" s="16"/>
       <c r="C62" s="16"/>
@@ -4491,7 +4505,7 @@
     </row>
     <row r="63" ht="15.0" customHeight="1">
       <c r="A63" s="17" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B63" s="18">
         <v>1090.43</v>
@@ -4511,7 +4525,7 @@
     </row>
     <row r="64" ht="15.0" customHeight="1">
       <c r="A64" s="14" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B64" s="15">
         <v>629.69</v>
@@ -4531,7 +4545,7 @@
     </row>
     <row r="65" ht="15.0" customHeight="1">
       <c r="A65" s="14" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B65" s="15">
         <v>1553.54</v>
@@ -4551,7 +4565,7 @@
     </row>
     <row r="66" ht="15.0" customHeight="1">
       <c r="A66" s="14" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B66" s="21">
         <v>10.63</v>
@@ -4571,27 +4585,27 @@
     </row>
     <row r="67" ht="15.0" customHeight="1">
       <c r="A67" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="B67" s="25">
+        <v>155</v>
+      </c>
+      <c r="B67" s="26">
         <v>-1611.43</v>
       </c>
-      <c r="C67" s="25">
+      <c r="C67" s="26">
         <v>-1613.25</v>
       </c>
-      <c r="D67" s="25">
+      <c r="D67" s="26">
         <v>-1474.19</v>
       </c>
-      <c r="E67" s="25">
+      <c r="E67" s="26">
         <v>-1200.45</v>
       </c>
-      <c r="F67" s="25">
+      <c r="F67" s="26">
         <v>-890.02</v>
       </c>
     </row>
     <row r="68" ht="15.0" customHeight="1">
       <c r="A68" s="14" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B68" s="21">
         <v>86.24</v>
@@ -4602,16 +4616,16 @@
       <c r="D68" s="20">
         <v>-59.28</v>
       </c>
-      <c r="E68" s="25">
+      <c r="E68" s="26">
         <v>-183.47</v>
       </c>
-      <c r="F68" s="25">
+      <c r="F68" s="26">
         <v>-257.3</v>
       </c>
     </row>
     <row r="69" ht="15.0" customHeight="1">
       <c r="A69" s="14" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B69" s="21">
         <v>1.18</v>
@@ -4627,7 +4641,7 @@
     </row>
     <row r="70" ht="15.0" customHeight="1">
       <c r="A70" s="17" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B70" s="18">
         <v>669.85</v>
@@ -4647,7 +4661,7 @@
     </row>
     <row r="71" ht="15.0" customHeight="1">
       <c r="A71" s="17" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B71" s="18">
         <v>669.85</v>
@@ -4667,7 +4681,7 @@
     </row>
     <row r="72" ht="15.0" customHeight="1">
       <c r="A72" s="14" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B72" s="16"/>
       <c r="C72" s="21">
@@ -4679,7 +4693,7 @@
     </row>
     <row r="73" ht="15.0" customHeight="1">
       <c r="A73" s="14" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B73" s="15">
         <v>141.77</v>
@@ -4699,7 +4713,7 @@
     </row>
     <row r="74" ht="15.0" customHeight="1">
       <c r="A74" s="14" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B74" s="16"/>
       <c r="C74" s="21">
@@ -4717,7 +4731,7 @@
     </row>
     <row r="75" ht="15.0" customHeight="1">
       <c r="A75" s="14" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B75" s="16"/>
       <c r="C75" s="16"/>
@@ -4731,7 +4745,7 @@
     </row>
     <row r="76" ht="15.0" customHeight="1">
       <c r="A76" s="14" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B76" s="16"/>
       <c r="C76" s="16"/>
@@ -4747,7 +4761,7 @@
     </row>
     <row r="77" ht="15.0" customHeight="1">
       <c r="A77" s="14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B77" s="16"/>
       <c r="C77" s="16"/>
@@ -4761,7 +4775,7 @@
     </row>
     <row r="78" ht="15.0" customHeight="1">
       <c r="A78" s="14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B78" s="16"/>
       <c r="C78" s="21">
@@ -4779,7 +4793,7 @@
     </row>
     <row r="79" ht="15.0" customHeight="1">
       <c r="A79" s="14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B79" s="16">
         <v>0.0</v>
@@ -4791,7 +4805,7 @@
     </row>
     <row r="80" ht="15.0" customHeight="1">
       <c r="A80" s="14" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B80" s="16"/>
       <c r="C80" s="16"/>
@@ -4807,7 +4821,7 @@
     </row>
     <row r="81" ht="15.0" customHeight="1">
       <c r="A81" s="14" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B81" s="21">
         <v>80.34</v>
@@ -4827,7 +4841,7 @@
     </row>
     <row r="82" ht="15.0" customHeight="1">
       <c r="A82" s="14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B82" s="21">
         <v>11.81</v>
@@ -4839,7 +4853,7 @@
     </row>
     <row r="83" ht="15.0" customHeight="1">
       <c r="A83" s="17" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B83" s="18">
         <v>233.92</v>
@@ -4859,7 +4873,7 @@
     </row>
     <row r="84" ht="15.0" customHeight="1">
       <c r="A84" s="14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B84" s="16"/>
       <c r="C84" s="21">
@@ -4871,7 +4885,7 @@
     </row>
     <row r="85" ht="15.0" customHeight="1">
       <c r="A85" s="14" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B85" s="16"/>
       <c r="C85" s="21">
@@ -4889,7 +4903,7 @@
     </row>
     <row r="86" ht="15.0" customHeight="1">
       <c r="A86" s="14" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B86" s="16"/>
       <c r="C86" s="21">
@@ -4901,7 +4915,7 @@
     </row>
     <row r="87" ht="15.0" customHeight="1">
       <c r="A87" s="14" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B87" s="21">
         <v>20.08</v>
@@ -4921,7 +4935,7 @@
     </row>
     <row r="88" ht="15.0" customHeight="1">
       <c r="A88" s="14" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B88" s="16"/>
       <c r="C88" s="16"/>
@@ -4935,7 +4949,7 @@
     </row>
     <row r="89" ht="15.0" customHeight="1">
       <c r="A89" s="14" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B89" s="16"/>
       <c r="C89" s="16"/>
@@ -4947,7 +4961,7 @@
     </row>
     <row r="90" ht="15.0" customHeight="1">
       <c r="A90" s="14" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B90" s="16"/>
       <c r="C90" s="16"/>
@@ -4959,7 +4973,7 @@
     </row>
     <row r="91" ht="15.0" customHeight="1">
       <c r="A91" s="14" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B91" s="21">
         <v>73.25</v>
@@ -4979,7 +4993,7 @@
     </row>
     <row r="92" ht="15.0" customHeight="1">
       <c r="A92" s="14" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B92" s="21">
         <v>48.44</v>
@@ -4999,7 +5013,7 @@
     </row>
     <row r="93" ht="15.0" customHeight="1">
       <c r="A93" s="14" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B93" s="21">
         <v>44.89</v>
@@ -5019,7 +5033,7 @@
     </row>
     <row r="94" ht="15.0" customHeight="1">
       <c r="A94" s="14" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B94" s="16"/>
       <c r="C94" s="21">
@@ -5037,7 +5051,7 @@
     </row>
     <row r="95" ht="15.0" customHeight="1">
       <c r="A95" s="17" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B95" s="18">
         <v>186.66</v>
@@ -5045,10 +5059,10 @@
       <c r="C95" s="18">
         <v>218.87</v>
       </c>
-      <c r="D95" s="22">
+      <c r="D95" s="23">
         <v>86.12</v>
       </c>
-      <c r="E95" s="22">
+      <c r="E95" s="23">
         <v>72.34</v>
       </c>
       <c r="F95" s="18">
@@ -5057,7 +5071,7 @@
     </row>
     <row r="96" ht="15.0" customHeight="1">
       <c r="A96" s="14" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B96" s="21">
         <v>10.63</v>
@@ -5069,7 +5083,7 @@
     </row>
     <row r="97" ht="15.0" customHeight="1">
       <c r="A97" s="14" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B97" s="16"/>
       <c r="C97" s="16"/>
@@ -5083,7 +5097,7 @@
     </row>
     <row r="98" ht="15.0" customHeight="1">
       <c r="A98" s="17" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B98" s="18">
         <v>431.21</v>
@@ -5103,7 +5117,7 @@
     </row>
     <row r="99" ht="15.0" customHeight="1">
       <c r="A99" s="14" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B99" s="20">
         <v>-10.63</v>
@@ -5115,7 +5129,7 @@
     </row>
     <row r="100" ht="15.0" customHeight="1">
       <c r="A100" s="17" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B100" s="18">
         <v>1090.43</v>
@@ -5135,7 +5149,7 @@
     </row>
     <row r="101" ht="15.0" customHeight="1">
       <c r="A101" s="14" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B101" s="21">
         <v>0.01</v>
@@ -5155,7 +5169,7 @@
     </row>
     <row r="102" ht="15.0" customHeight="1">
       <c r="A102" s="14" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B102" s="21">
         <v>11.97</v>
@@ -5175,7 +5189,7 @@
     </row>
     <row r="103" ht="15.0" customHeight="1">
       <c r="A103" s="14" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B103" s="21">
         <v>11.97</v>
@@ -5195,7 +5209,7 @@
     </row>
     <row r="104" ht="15.0" customHeight="1">
       <c r="A104" s="14" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B104" s="16"/>
       <c r="C104" s="15">
@@ -5207,7 +5221,7 @@
     </row>
     <row r="105" ht="15.0" customHeight="1">
       <c r="A105" s="14" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B105" s="16"/>
       <c r="C105" s="15">
@@ -5219,7 +5233,7 @@
     </row>
     <row r="106" ht="15.0" customHeight="1">
       <c r="A106" s="14" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B106" s="16"/>
       <c r="C106" s="15">
@@ -5231,7 +5245,7 @@
     </row>
     <row r="107" ht="15.0" customHeight="1">
       <c r="A107" s="14" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B107" s="16"/>
       <c r="C107" s="16">
@@ -5243,7 +5257,7 @@
     </row>
     <row r="108" ht="15.0" customHeight="1">
       <c r="A108" s="14" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B108" s="21">
         <v>11.97</v>
@@ -5263,7 +5277,7 @@
     </row>
     <row r="109" ht="15.0" customHeight="1">
       <c r="A109" s="14" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B109" s="21">
         <v>0.01</v>
@@ -5283,7 +5297,7 @@
     </row>
     <row r="110" ht="15.0" customHeight="1">
       <c r="A110" s="14" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B110" s="21">
         <v>11.97</v>
@@ -5303,7 +5317,7 @@
     </row>
     <row r="111" ht="15.0" customHeight="1">
       <c r="A111" s="14" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B111" s="21">
         <v>1.0</v>
@@ -5323,7 +5337,7 @@
     </row>
     <row r="112" ht="15.0" customHeight="1">
       <c r="A112" s="14" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B112" s="21">
         <v>84.0</v>
@@ -6245,7 +6259,7 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -6410,19 +6424,19 @@
         <v>27</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="16" ht="15.0" customHeight="1" outlineLevel="1">
@@ -6447,7 +6461,7 @@
     </row>
     <row r="18">
       <c r="A18" s="12" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -6477,7 +6491,7 @@
     </row>
     <row r="20" ht="15.0" customHeight="1">
       <c r="A20" s="14" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B20" s="21">
         <v>85.43</v>
@@ -6488,16 +6502,16 @@
       <c r="D20" s="20">
         <v>-60.46</v>
       </c>
-      <c r="E20" s="25">
+      <c r="E20" s="26">
         <v>-176.64</v>
       </c>
-      <c r="F20" s="25">
+      <c r="F20" s="26">
         <v>-261.16</v>
       </c>
     </row>
     <row r="21" ht="15.0" customHeight="1">
       <c r="A21" s="14" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B21" s="21">
         <v>71.39</v>
@@ -6535,7 +6549,7 @@
     </row>
     <row r="23" ht="15.0" customHeight="1">
       <c r="A23" s="14" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B23" s="16"/>
       <c r="C23" s="16"/>
@@ -6547,7 +6561,7 @@
     </row>
     <row r="24" ht="15.0" customHeight="1">
       <c r="A24" s="14" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B24" s="20">
         <v>-24.58</v>
@@ -6567,7 +6581,7 @@
     </row>
     <row r="25" ht="15.0" customHeight="1">
       <c r="A25" s="14" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B25" s="20">
         <v>-47.98</v>
@@ -6587,7 +6601,7 @@
     </row>
     <row r="26" ht="15.0" customHeight="1">
       <c r="A26" s="14" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B26" s="15">
         <v>186.07</v>
@@ -6601,13 +6615,13 @@
       <c r="E26" s="20">
         <v>-68.64</v>
       </c>
-      <c r="F26" s="25">
+      <c r="F26" s="26">
         <v>-110.76</v>
       </c>
     </row>
     <row r="27" ht="15.0" customHeight="1">
       <c r="A27" s="14" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B27" s="20">
         <v>-57.34</v>
@@ -6627,7 +6641,7 @@
     </row>
     <row r="28" ht="15.0" customHeight="1">
       <c r="A28" s="14" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B28" s="20">
         <v>-9.36</v>
@@ -6647,7 +6661,7 @@
     </row>
     <row r="29" ht="15.0" customHeight="1">
       <c r="A29" s="14" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B29" s="21">
         <v>39.79</v>
@@ -6667,7 +6681,7 @@
     </row>
     <row r="30" ht="15.0" customHeight="1">
       <c r="A30" s="14" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B30" s="20">
         <v>-25.75</v>
@@ -6687,7 +6701,7 @@
     </row>
     <row r="31" ht="15.0" customHeight="1">
       <c r="A31" s="14" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B31" s="20">
         <v>-8.19</v>
@@ -6707,7 +6721,7 @@
     </row>
     <row r="32" ht="15.0" customHeight="1">
       <c r="A32" s="14" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B32" s="16">
         <v>0.0</v>
@@ -6723,7 +6737,7 @@
     </row>
     <row r="33" ht="15.0" customHeight="1">
       <c r="A33" s="14" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B33" s="21">
         <v>2.34</v>
@@ -6741,27 +6755,27 @@
     </row>
     <row r="34" ht="15.0" customHeight="1">
       <c r="A34" s="17" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B34" s="18">
         <v>153.3</v>
       </c>
-      <c r="C34" s="22">
+      <c r="C34" s="23">
         <v>72.04</v>
       </c>
-      <c r="D34" s="23">
+      <c r="D34" s="24">
         <v>-34.22</v>
       </c>
-      <c r="E34" s="23">
+      <c r="E34" s="24">
         <v>-48.45</v>
       </c>
-      <c r="F34" s="24">
+      <c r="F34" s="25">
         <v>-108.73</v>
       </c>
     </row>
     <row r="35" ht="15.0" customHeight="1">
       <c r="A35" s="14" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B35" s="20">
         <v>-50.32</v>
@@ -6781,9 +6795,9 @@
     </row>
     <row r="36" ht="15.0" customHeight="1">
       <c r="A36" s="14" t="s">
-        <v>217</v>
-      </c>
-      <c r="B36" s="25">
+        <v>218</v>
+      </c>
+      <c r="B36" s="26">
         <v>-154.47</v>
       </c>
       <c r="C36" s="20">
@@ -6801,7 +6815,7 @@
     </row>
     <row r="37" ht="15.0" customHeight="1">
       <c r="A37" s="14" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B37" s="16">
         <v>0.0</v>
@@ -6817,7 +6831,7 @@
     </row>
     <row r="38" ht="15.0" customHeight="1">
       <c r="A38" s="14" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B38" s="20">
         <v>-10.53</v>
@@ -6829,7 +6843,7 @@
     </row>
     <row r="39" ht="15.0" customHeight="1">
       <c r="A39" s="14" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B39" s="21">
         <v>1.17</v>
@@ -6843,27 +6857,27 @@
     </row>
     <row r="40" ht="15.0" customHeight="1">
       <c r="A40" s="17" t="s">
-        <v>221</v>
-      </c>
-      <c r="B40" s="24">
+        <v>222</v>
+      </c>
+      <c r="B40" s="25">
         <v>-214.16</v>
       </c>
-      <c r="C40" s="24">
+      <c r="C40" s="25">
         <v>-118.52</v>
       </c>
-      <c r="D40" s="23">
+      <c r="D40" s="24">
         <v>-79.85</v>
       </c>
-      <c r="E40" s="23">
+      <c r="E40" s="24">
         <v>-32.3</v>
       </c>
-      <c r="F40" s="23">
+      <c r="F40" s="24">
         <v>-49.79</v>
       </c>
     </row>
     <row r="41" ht="15.0" customHeight="1">
       <c r="A41" s="14" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
@@ -6879,7 +6893,7 @@
     </row>
     <row r="42" ht="15.0" customHeight="1">
       <c r="A42" s="14" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B42" s="16"/>
       <c r="C42" s="16"/>
@@ -6895,7 +6909,7 @@
     </row>
     <row r="43" ht="15.0" customHeight="1">
       <c r="A43" s="14" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B43" s="21">
         <v>86.6</v>
@@ -6915,7 +6929,7 @@
     </row>
     <row r="44" ht="15.0" customHeight="1">
       <c r="A44" s="14" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B44" s="20">
         <v>-3.51</v>
@@ -6929,13 +6943,13 @@
       <c r="E44" s="20">
         <v>-66.62</v>
       </c>
-      <c r="F44" s="25">
+      <c r="F44" s="26">
         <v>-126.0</v>
       </c>
     </row>
     <row r="45" ht="15.0" customHeight="1">
       <c r="A45" s="14" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B45" s="16">
         <v>0.0</v>
@@ -6955,7 +6969,7 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="A46" s="14" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B46" s="20">
         <v>-1.17</v>
@@ -6971,15 +6985,15 @@
     </row>
     <row r="47" ht="15.0" customHeight="1">
       <c r="A47" s="17" t="s">
-        <v>228</v>
-      </c>
-      <c r="B47" s="22">
+        <v>229</v>
+      </c>
+      <c r="B47" s="23">
         <v>81.92</v>
       </c>
-      <c r="C47" s="22">
+      <c r="C47" s="23">
         <v>56.94</v>
       </c>
-      <c r="D47" s="22">
+      <c r="D47" s="23">
         <v>85.56</v>
       </c>
       <c r="E47" s="18">
@@ -6991,7 +7005,7 @@
     </row>
     <row r="48" ht="15.0" customHeight="1">
       <c r="A48" s="14" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B48" s="16">
         <v>0.0</v>
@@ -7007,7 +7021,7 @@
     </row>
     <row r="49" ht="15.0" customHeight="1">
       <c r="A49" s="14" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B49" s="21">
         <v>24.81</v>
@@ -7027,7 +7041,7 @@
     </row>
     <row r="50" ht="15.0" customHeight="1">
       <c r="A50" s="14" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B50" s="21">
         <v>46.07</v>
@@ -7047,7 +7061,7 @@
     </row>
     <row r="51" ht="15.0" customHeight="1">
       <c r="A51" s="14" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B51" s="21">
         <v>21.06</v>
@@ -7067,21 +7081,21 @@
     </row>
     <row r="52" ht="15.0" customHeight="1">
       <c r="A52" s="17" t="s">
-        <v>233</v>
-      </c>
-      <c r="B52" s="22">
+        <v>234</v>
+      </c>
+      <c r="B52" s="23">
         <v>21.06</v>
       </c>
-      <c r="C52" s="22">
+      <c r="C52" s="23">
         <v>10.46</v>
       </c>
-      <c r="D52" s="23">
+      <c r="D52" s="24">
         <v>-28.52</v>
       </c>
-      <c r="E52" s="22">
+      <c r="E52" s="23">
         <v>25.23</v>
       </c>
-      <c r="F52" s="22">
+      <c r="F52" s="23">
         <v>1.02</v>
       </c>
     </row>
@@ -8055,7 +8069,7 @@
   <sheetData>
     <row r="1" ht="15.0" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -8238,7 +8252,7 @@
     </row>
     <row r="18">
       <c r="A18" s="12" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -8263,353 +8277,353 @@
       </c>
     </row>
     <row r="20" ht="15.0" customHeight="1">
-      <c r="A20" s="26" t="s">
-        <v>236</v>
-      </c>
-      <c r="B20" s="27"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
+      <c r="A20" s="27" t="s">
+        <v>237</v>
+      </c>
+      <c r="B20" s="28"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
     </row>
     <row r="21" ht="15.0" customHeight="1">
-      <c r="A21" s="28" t="s">
-        <v>236</v>
-      </c>
-      <c r="B21" s="29">
+      <c r="A21" s="29" t="s">
+        <v>237</v>
+      </c>
+      <c r="B21" s="30">
         <v>1516.24</v>
       </c>
-      <c r="C21" s="29">
+      <c r="C21" s="30">
         <v>824.02</v>
       </c>
-      <c r="D21" s="29">
+      <c r="D21" s="30">
         <v>559.23</v>
       </c>
-      <c r="E21" s="30"/>
+      <c r="E21" s="31"/>
     </row>
     <row r="22" ht="15.0" customHeight="1">
-      <c r="A22" s="26" t="s">
-        <v>237</v>
-      </c>
-      <c r="B22" s="27"/>
-      <c r="C22" s="27"/>
-      <c r="D22" s="27"/>
-      <c r="E22" s="27"/>
+      <c r="A22" s="27" t="s">
+        <v>238</v>
+      </c>
+      <c r="B22" s="28"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
     </row>
     <row r="23" ht="15.0" customHeight="1">
-      <c r="A23" s="28" t="s">
-        <v>237</v>
-      </c>
-      <c r="B23" s="29">
+      <c r="A23" s="29" t="s">
+        <v>238</v>
+      </c>
+      <c r="B23" s="30">
         <v>1052.63</v>
       </c>
-      <c r="C23" s="29">
+      <c r="C23" s="30">
         <v>657.37</v>
       </c>
-      <c r="D23" s="29">
+      <c r="D23" s="30">
         <v>486.89</v>
       </c>
-      <c r="E23" s="30"/>
+      <c r="E23" s="31"/>
     </row>
     <row r="24" ht="15.0" customHeight="1">
-      <c r="A24" s="26" t="s">
-        <v>238</v>
-      </c>
-      <c r="B24" s="27"/>
-      <c r="C24" s="27"/>
-      <c r="D24" s="27"/>
-      <c r="E24" s="27"/>
+      <c r="A24" s="27" t="s">
+        <v>239</v>
+      </c>
+      <c r="B24" s="28"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28"/>
     </row>
     <row r="25" ht="15.0" customHeight="1">
-      <c r="A25" s="28" t="s">
-        <v>239</v>
-      </c>
-      <c r="B25" s="31">
+      <c r="A25" s="29" t="s">
+        <v>240</v>
+      </c>
+      <c r="B25" s="32">
         <v>97.2</v>
       </c>
-      <c r="C25" s="31">
+      <c r="C25" s="32">
         <v>67.11</v>
       </c>
-      <c r="D25" s="31">
+      <c r="D25" s="32">
         <v>52.42</v>
       </c>
-      <c r="E25" s="30"/>
+      <c r="E25" s="31"/>
     </row>
     <row r="26" ht="15.0" customHeight="1">
-      <c r="A26" s="26" t="s">
-        <v>240</v>
-      </c>
-      <c r="B26" s="27"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="27"/>
-      <c r="E26" s="27"/>
+      <c r="A26" s="27" t="s">
+        <v>241</v>
+      </c>
+      <c r="B26" s="28"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="28"/>
+      <c r="E26" s="28"/>
     </row>
     <row r="27" ht="15.0" customHeight="1">
-      <c r="A27" s="28" t="s">
-        <v>241</v>
-      </c>
-      <c r="B27" s="32">
+      <c r="A27" s="29" t="s">
+        <v>242</v>
+      </c>
+      <c r="B27" s="33">
         <v>-5.04</v>
       </c>
-      <c r="C27" s="32">
+      <c r="C27" s="33">
         <v>-17.56</v>
       </c>
-      <c r="D27" s="32">
+      <c r="D27" s="33">
         <v>-17.23</v>
       </c>
-      <c r="E27" s="33"/>
+      <c r="E27" s="34"/>
     </row>
     <row r="28" ht="15.0" customHeight="1">
-      <c r="A28" s="26" t="s">
-        <v>242</v>
-      </c>
-      <c r="B28" s="27"/>
-      <c r="C28" s="27"/>
-      <c r="D28" s="27"/>
-      <c r="E28" s="27"/>
+      <c r="A28" s="27" t="s">
+        <v>243</v>
+      </c>
+      <c r="B28" s="28"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="28"/>
     </row>
     <row r="29" ht="15.0" customHeight="1">
-      <c r="A29" s="28" t="s">
-        <v>243</v>
-      </c>
-      <c r="B29" s="33">
+      <c r="A29" s="29" t="s">
+        <v>244</v>
+      </c>
+      <c r="B29" s="34">
         <v>0.0</v>
       </c>
-      <c r="C29" s="33">
+      <c r="C29" s="34">
         <v>0.0</v>
       </c>
-      <c r="D29" s="33">
+      <c r="D29" s="34">
         <v>0.0</v>
       </c>
-      <c r="E29" s="33"/>
+      <c r="E29" s="34"/>
     </row>
     <row r="30" ht="15.0" customHeight="1">
-      <c r="A30" s="28" t="s">
-        <v>244</v>
-      </c>
-      <c r="B30" s="33">
+      <c r="A30" s="29" t="s">
+        <v>245</v>
+      </c>
+      <c r="B30" s="34">
         <v>0.0</v>
       </c>
-      <c r="C30" s="33">
+      <c r="C30" s="34">
         <v>0.0</v>
       </c>
-      <c r="D30" s="33">
+      <c r="D30" s="34">
         <v>0.0</v>
       </c>
-      <c r="E30" s="33"/>
+      <c r="E30" s="34"/>
     </row>
     <row r="31" ht="15.0" customHeight="1">
-      <c r="A31" s="26" t="s">
-        <v>245</v>
-      </c>
-      <c r="B31" s="27"/>
-      <c r="C31" s="27"/>
-      <c r="D31" s="27"/>
-      <c r="E31" s="27"/>
+      <c r="A31" s="27" t="s">
+        <v>246</v>
+      </c>
+      <c r="B31" s="28"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="28"/>
     </row>
     <row r="32" ht="15.0" customHeight="1">
-      <c r="A32" s="28" t="s">
-        <v>246</v>
-      </c>
-      <c r="B32" s="31">
+      <c r="A32" s="29" t="s">
+        <v>247</v>
+      </c>
+      <c r="B32" s="32">
         <v>2.17</v>
       </c>
-      <c r="C32" s="31">
+      <c r="C32" s="32">
         <v>1.72</v>
       </c>
-      <c r="D32" s="31">
+      <c r="D32" s="32">
         <v>1.28</v>
       </c>
-      <c r="E32" s="30"/>
+      <c r="E32" s="31"/>
     </row>
     <row r="33" ht="15.0" customHeight="1">
-      <c r="A33" s="26" t="s">
-        <v>247</v>
-      </c>
-      <c r="B33" s="27"/>
-      <c r="C33" s="27"/>
-      <c r="D33" s="27"/>
-      <c r="E33" s="27"/>
+      <c r="A33" s="27" t="s">
+        <v>248</v>
+      </c>
+      <c r="B33" s="28"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
     </row>
     <row r="34" ht="15.0" customHeight="1">
-      <c r="A34" s="28" t="s">
-        <v>248</v>
-      </c>
-      <c r="B34" s="31">
+      <c r="A34" s="29" t="s">
+        <v>249</v>
+      </c>
+      <c r="B34" s="32">
         <v>89.41</v>
       </c>
-      <c r="C34" s="30"/>
-      <c r="D34" s="31">
+      <c r="C34" s="31"/>
+      <c r="D34" s="32">
         <v>16.57</v>
       </c>
-      <c r="E34" s="30"/>
+      <c r="E34" s="31"/>
     </row>
     <row r="35" ht="15.0" customHeight="1">
-      <c r="A35" s="26" t="s">
-        <v>249</v>
-      </c>
-      <c r="B35" s="27"/>
-      <c r="C35" s="27"/>
-      <c r="D35" s="27"/>
-      <c r="E35" s="27"/>
+      <c r="A35" s="27" t="s">
+        <v>250</v>
+      </c>
+      <c r="B35" s="28"/>
+      <c r="C35" s="28"/>
+      <c r="D35" s="28"/>
+      <c r="E35" s="28"/>
     </row>
     <row r="36" ht="15.0" customHeight="1">
-      <c r="A36" s="28" t="s">
-        <v>250</v>
-      </c>
-      <c r="B36" s="31">
+      <c r="A36" s="29" t="s">
+        <v>251</v>
+      </c>
+      <c r="B36" s="32">
         <v>2.84</v>
       </c>
-      <c r="C36" s="31">
+      <c r="C36" s="32">
         <v>2.92</v>
       </c>
-      <c r="D36" s="31">
+      <c r="D36" s="32">
         <v>3.44</v>
       </c>
-      <c r="E36" s="30"/>
+      <c r="E36" s="31"/>
     </row>
     <row r="37" ht="15.0" customHeight="1">
-      <c r="A37" s="26" t="s">
-        <v>251</v>
-      </c>
-      <c r="B37" s="27"/>
-      <c r="C37" s="27"/>
-      <c r="D37" s="27"/>
-      <c r="E37" s="27"/>
+      <c r="A37" s="27" t="s">
+        <v>252</v>
+      </c>
+      <c r="B37" s="28"/>
+      <c r="C37" s="28"/>
+      <c r="D37" s="28"/>
+      <c r="E37" s="28"/>
     </row>
     <row r="38" ht="15.0" customHeight="1">
-      <c r="A38" s="28" t="s">
-        <v>252</v>
-      </c>
-      <c r="B38" s="31">
+      <c r="A38" s="29" t="s">
+        <v>253</v>
+      </c>
+      <c r="B38" s="32">
         <v>2.37</v>
       </c>
-      <c r="C38" s="30"/>
-      <c r="D38" s="30"/>
-      <c r="E38" s="30"/>
+      <c r="C38" s="31"/>
+      <c r="D38" s="31"/>
+      <c r="E38" s="31"/>
     </row>
     <row r="39" ht="15.0" customHeight="1">
-      <c r="A39" s="26" t="s">
-        <v>253</v>
-      </c>
-      <c r="B39" s="27"/>
-      <c r="C39" s="27"/>
-      <c r="D39" s="27"/>
-      <c r="E39" s="27"/>
+      <c r="A39" s="27" t="s">
+        <v>254</v>
+      </c>
+      <c r="B39" s="28"/>
+      <c r="C39" s="28"/>
+      <c r="D39" s="28"/>
+      <c r="E39" s="28"/>
     </row>
     <row r="40" ht="15.0" customHeight="1">
-      <c r="A40" s="28" t="s">
-        <v>254</v>
-      </c>
-      <c r="B40" s="29">
+      <c r="A40" s="29" t="s">
+        <v>255</v>
+      </c>
+      <c r="B40" s="30">
         <v>271.26</v>
       </c>
-      <c r="C40" s="30"/>
-      <c r="D40" s="30"/>
-      <c r="E40" s="30"/>
+      <c r="C40" s="31"/>
+      <c r="D40" s="31"/>
+      <c r="E40" s="31"/>
     </row>
     <row r="41" ht="15.0" customHeight="1">
-      <c r="A41" s="26" t="s">
-        <v>255</v>
-      </c>
-      <c r="B41" s="27"/>
-      <c r="C41" s="27"/>
-      <c r="D41" s="27"/>
-      <c r="E41" s="27"/>
+      <c r="A41" s="27" t="s">
+        <v>256</v>
+      </c>
+      <c r="B41" s="28"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="28"/>
+      <c r="E41" s="28"/>
     </row>
     <row r="42" ht="15.0" customHeight="1">
-      <c r="A42" s="28" t="s">
-        <v>256</v>
-      </c>
-      <c r="B42" s="29">
+      <c r="A42" s="29" t="s">
+        <v>257</v>
+      </c>
+      <c r="B42" s="30">
         <v>271.26</v>
       </c>
-      <c r="C42" s="30"/>
-      <c r="D42" s="30"/>
-      <c r="E42" s="30"/>
+      <c r="C42" s="31"/>
+      <c r="D42" s="31"/>
+      <c r="E42" s="31"/>
     </row>
     <row r="43" ht="15.0" customHeight="1">
-      <c r="A43" s="26" t="s">
-        <v>257</v>
-      </c>
-      <c r="B43" s="27"/>
-      <c r="C43" s="27"/>
-      <c r="D43" s="27"/>
-      <c r="E43" s="27"/>
+      <c r="A43" s="27" t="s">
+        <v>258</v>
+      </c>
+      <c r="B43" s="28"/>
+      <c r="C43" s="28"/>
+      <c r="D43" s="28"/>
+      <c r="E43" s="28"/>
     </row>
     <row r="44" ht="15.0" customHeight="1">
-      <c r="A44" s="28" t="s">
-        <v>258</v>
-      </c>
-      <c r="B44" s="31">
+      <c r="A44" s="29" t="s">
+        <v>259</v>
+      </c>
+      <c r="B44" s="32">
         <v>2.57</v>
       </c>
-      <c r="C44" s="30"/>
-      <c r="D44" s="30"/>
-      <c r="E44" s="30"/>
+      <c r="C44" s="31"/>
+      <c r="D44" s="31"/>
+      <c r="E44" s="31"/>
     </row>
     <row r="45" ht="15.0" customHeight="1">
-      <c r="A45" s="26" t="s">
-        <v>259</v>
-      </c>
-      <c r="B45" s="27"/>
-      <c r="C45" s="27"/>
-      <c r="D45" s="27"/>
-      <c r="E45" s="27"/>
+      <c r="A45" s="27" t="s">
+        <v>260</v>
+      </c>
+      <c r="B45" s="28"/>
+      <c r="C45" s="28"/>
+      <c r="D45" s="28"/>
+      <c r="E45" s="28"/>
     </row>
     <row r="46" ht="15.0" customHeight="1">
-      <c r="A46" s="28" t="s">
-        <v>260</v>
-      </c>
-      <c r="B46" s="31">
+      <c r="A46" s="29" t="s">
+        <v>261</v>
+      </c>
+      <c r="B46" s="32">
         <v>4.49</v>
       </c>
-      <c r="C46" s="31">
+      <c r="C46" s="32">
         <v>3.74</v>
       </c>
-      <c r="D46" s="31">
+      <c r="D46" s="32">
         <v>3.95</v>
       </c>
-      <c r="E46" s="30"/>
+      <c r="E46" s="31"/>
     </row>
     <row r="47" ht="15.0" customHeight="1">
-      <c r="A47" s="26" t="s">
-        <v>261</v>
-      </c>
-      <c r="B47" s="27"/>
-      <c r="C47" s="27"/>
-      <c r="D47" s="27"/>
-      <c r="E47" s="27"/>
+      <c r="A47" s="27" t="s">
+        <v>262</v>
+      </c>
+      <c r="B47" s="28"/>
+      <c r="C47" s="28"/>
+      <c r="D47" s="28"/>
+      <c r="E47" s="28"/>
     </row>
     <row r="48" ht="15.0" customHeight="1">
-      <c r="A48" s="28" t="s">
-        <v>262</v>
-      </c>
-      <c r="B48" s="31">
+      <c r="A48" s="29" t="s">
+        <v>263</v>
+      </c>
+      <c r="B48" s="32">
         <v>3.52</v>
       </c>
-      <c r="C48" s="30"/>
-      <c r="D48" s="30"/>
-      <c r="E48" s="30"/>
+      <c r="C48" s="31"/>
+      <c r="D48" s="31"/>
+      <c r="E48" s="31"/>
     </row>
     <row r="49" ht="15.0" customHeight="1">
-      <c r="A49" s="26" t="s">
-        <v>263</v>
-      </c>
-      <c r="B49" s="27"/>
-      <c r="C49" s="27"/>
-      <c r="D49" s="27"/>
-      <c r="E49" s="27"/>
+      <c r="A49" s="27" t="s">
+        <v>264</v>
+      </c>
+      <c r="B49" s="28"/>
+      <c r="C49" s="28"/>
+      <c r="D49" s="28"/>
+      <c r="E49" s="28"/>
     </row>
     <row r="50" ht="15.0" customHeight="1">
-      <c r="A50" s="28" t="s">
-        <v>264</v>
-      </c>
-      <c r="B50" s="31">
+      <c r="A50" s="29" t="s">
+        <v>265</v>
+      </c>
+      <c r="B50" s="32">
         <v>20.78</v>
       </c>
-      <c r="C50" s="30"/>
-      <c r="D50" s="30"/>
-      <c r="E50" s="30"/>
+      <c r="C50" s="31"/>
+      <c r="D50" s="31"/>
+      <c r="E50" s="31"/>
     </row>
     <row r="51" ht="15.75" customHeight="1"/>
     <row r="52" ht="15.75" customHeight="1"/>

</xml_diff>